<commit_message>
QA & Development Practical Assessment
</commit_message>
<xml_diff>
--- a/QA & Development Practical Assessment .xlsx
+++ b/QA & Development Practical Assessment .xlsx
@@ -5,18 +5,16 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930" firstSheet="1" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" firstSheet="1" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="T1P1-Test Strategy" sheetId="1" r:id="rId1"/>
     <sheet name="T1P2-Practical Testing" sheetId="2" r:id="rId2"/>
     <sheet name="T1P3-Risk Analysis " sheetId="3" r:id="rId3"/>
-    <sheet name="T1P4-Automation " sheetId="5" r:id="rId4"/>
-    <sheet name="T2-Unit Testing" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="143">
   <si>
     <t>Expected Result</t>
   </si>
@@ -474,19 +472,13 @@
   </si>
   <si>
     <t>The bar's color isn't responsive.</t>
-  </si>
-  <si>
-    <t>It got attached to zip file</t>
-  </si>
-  <si>
-    <t>As a software tester, I possess strong expertise in validating and ensuring the quality of existing web services. While I have not yet gained hands-on experience in developing web services from the ground up, I am fully capable of performing comprehensive testing across functional, performance, and security dimensions. At this stage in my career, my focus remains on testing and quality assurance rather than service development, though I remain open to expanding my skill set in the future.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -531,14 +523,6 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="4"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -796,7 +780,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -897,12 +881,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1531,22 +1509,22 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="15.36328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.26953125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="42.6328125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="44.6328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.08984375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="59.90625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="39.36328125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="26.1796875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="9.26953125" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" style="2"/>
+    <col min="1" max="1" width="13.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.21875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="42.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="44.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="59.88671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="39.33203125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="26.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="9.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.77734375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="23" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
@@ -1578,7 +1556,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
         <v>30</v>
       </c>
@@ -1610,7 +1588,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>31</v>
       </c>
@@ -1642,7 +1620,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>32</v>
       </c>
@@ -1674,7 +1652,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>33</v>
       </c>
@@ -1706,7 +1684,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>34</v>
       </c>
@@ -1738,7 +1716,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>35</v>
       </c>
@@ -1770,7 +1748,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>36</v>
       </c>
@@ -1802,7 +1780,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>37</v>
       </c>
@@ -1834,7 +1812,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>38</v>
       </c>
@@ -1866,7 +1844,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>39</v>
       </c>
@@ -1898,7 +1876,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>40</v>
       </c>
@@ -1930,7 +1908,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>41</v>
       </c>
@@ -1962,7 +1940,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>104</v>
       </c>
@@ -1994,7 +1972,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>112</v>
       </c>
@@ -2039,19 +2017,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.453125" customWidth="1"/>
-    <col min="2" max="2" width="45.1796875" customWidth="1"/>
+    <col min="1" max="1" width="28.44140625" customWidth="1"/>
+    <col min="2" max="2" width="45.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="33" t="s">
         <v>139</v>
       </c>
       <c r="B1" s="34"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
         <v>19</v>
       </c>
@@ -2059,7 +2037,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>20</v>
       </c>
@@ -2067,7 +2045,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="23" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="30" t="s">
         <v>21</v>
       </c>
@@ -2075,19 +2053,19 @@
         <v>129</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="31"/>
       <c r="B5" s="13" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="32"/>
       <c r="B6" s="13" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
         <v>126</v>
       </c>
@@ -2095,7 +2073,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="23" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
         <v>0</v>
       </c>
@@ -2103,7 +2081,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="23" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
         <v>1</v>
       </c>
@@ -2111,13 +2089,13 @@
         <v>132</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="124.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
         <v>22</v>
       </c>
       <c r="B10" s="28"/>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
         <v>23</v>
       </c>
@@ -2125,7 +2103,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
         <v>9</v>
       </c>
@@ -2133,7 +2111,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
         <v>24</v>
       </c>
@@ -2141,7 +2119,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
         <v>25</v>
       </c>
@@ -2149,7 +2127,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
         <v>26</v>
       </c>
@@ -2157,7 +2135,7 @@
         <v>45974</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="14" t="s">
         <v>27</v>
       </c>
@@ -2165,7 +2143,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
         <v>29</v>
       </c>
@@ -2173,17 +2151,17 @@
         <v>122</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="6.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" ht="6.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="29"/>
       <c r="B18" s="29"/>
     </row>
-    <row r="19" spans="1:2" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33" t="s">
         <v>140</v>
       </c>
       <c r="B19" s="34"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
         <v>19</v>
       </c>
@@ -2191,7 +2169,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="14" t="s">
         <v>20</v>
       </c>
@@ -2199,7 +2177,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="30" t="s">
         <v>21</v>
       </c>
@@ -2207,19 +2185,19 @@
         <v>129</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="31"/>
       <c r="B23" s="13" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="32"/>
       <c r="B24" s="13" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
         <v>126</v>
       </c>
@@ -2227,7 +2205,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="14" t="s">
         <v>0</v>
       </c>
@@ -2235,7 +2213,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="23" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A27" s="25" t="s">
         <v>1</v>
       </c>
@@ -2243,13 +2221,13 @@
         <v>132</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="162.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" ht="162.44999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="25" t="s">
         <v>22</v>
       </c>
       <c r="B28" s="28"/>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="14" t="s">
         <v>23</v>
       </c>
@@ -2257,7 +2235,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="14" t="s">
         <v>9</v>
       </c>
@@ -2265,7 +2243,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
         <v>24</v>
       </c>
@@ -2273,7 +2251,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
         <v>25</v>
       </c>
@@ -2281,7 +2259,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
         <v>26</v>
       </c>
@@ -2289,7 +2267,7 @@
         <v>45974</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
         <v>27</v>
       </c>
@@ -2297,7 +2275,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="14" t="s">
         <v>29</v>
       </c>
@@ -2320,32 +2298,32 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="89.453125" customWidth="1"/>
+    <col min="1" max="1" width="89.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="35.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" ht="35.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" ht="33.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
         <v>121</v>
       </c>
@@ -2357,41 +2335,4 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="43.81640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="36" t="s">
-        <v>143</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="82.90625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" ht="136" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="35" t="s">
-        <v>144</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>